<commit_message>
fixed a bunch of bugs in the code. Still need to go back and reorganize, make more reproducible.
</commit_message>
<xml_diff>
--- a/raw_data/metadata.xlsx
+++ b/raw_data/metadata.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10114"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10322"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/joegunn/Desktop/Projects/completed_projects/SNOLH_Genomics/raw_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73924601-35BD-BE45-81C5-9B6456AE4EF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE1C2A39-CB97-714A-9614-5F98E2FF430C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1160" yWindow="500" windowWidth="27640" windowHeight="15980" xr2:uid="{A65F9020-AEF3-134F-925A-DBC4100CC07D}"/>
+    <workbookView xWindow="12440" yWindow="500" windowWidth="27640" windowHeight="15980" xr2:uid="{A65F9020-AEF3-134F-925A-DBC4100CC07D}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -8649,10 +8649,10 @@
     <t>genetics_number</t>
   </si>
   <si>
-    <t>structure_nubmer</t>
-  </si>
-  <si>
     <t>putative_taxon</t>
+  </si>
+  <si>
+    <t>structure_number</t>
   </si>
 </sst>
 </file>
@@ -8802,9 +8802,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -8842,7 +8842,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -8948,7 +8948,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -9090,7 +9090,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -9125,7 +9125,7 @@
         <v>1186</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>1195</v>
+        <v>1194</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>1187</v>
@@ -9149,7 +9149,7 @@
         <v>1193</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>1194</v>
+        <v>1195</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.2">

</xml_diff>